<commit_message>
modified some issues in memory
</commit_message>
<xml_diff>
--- a/apartments.xlsx
+++ b/apartments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOQ\Documents\GitHub\Apartment-Recommendation-Chatbot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9361FBCF-94D5-4E4E-B0A3-D97432F7E6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9A5ADE-E6E0-403E-B4FC-2F0D17657FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="424">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="425">
   <si>
     <t>apartment_id</t>
   </si>
@@ -1292,6 +1292,9 @@
   </si>
   <si>
     <t>Duplex in MV iCity with premium lagoon-facing unit.</t>
+  </si>
+  <si>
+    <t>dadakiem2452001@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -2079,8 +2082,8 @@
       <c r="L2" t="s">
         <v>20</v>
       </c>
-      <c r="M2" t="s">
-        <v>21</v>
+      <c r="M2" s="1" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -5737,6 +5740,7 @@
     <hyperlink ref="M51" r:id="rId1" xr:uid="{9A50B3B0-D05F-40DB-B893-E99BF185BA59}"/>
     <hyperlink ref="M52:M71" r:id="rId2" display="ahmedashraf2452001@gmail.com" xr:uid="{F172BF1B-03FA-4436-9600-7978C2D52A23}"/>
     <hyperlink ref="M72:M91" r:id="rId3" display="ahmedashraf2452001@gmail.com" xr:uid="{3EC1D6A5-779A-4BB9-8C63-0E2A9F2FFECC}"/>
+    <hyperlink ref="M2" r:id="rId4" xr:uid="{3BB6CCD0-2FE0-4336-8EE6-4028F0FE9F8B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>